<commit_message>
feat: agrega consulta CPE via API SUNAT, plan de cuentas, auditoria y gestion de PDFs
Incorpora la API oficial consultacpe de SUNAT (XML/PDF) como via principal para
obtener el detalle y PDF de comprobantes, con el scraping Playwright como
respaldo automatico si la API falla. Suma modulos nuevos de plan de cuentas,
auditoria de cobertura y almacenamiento/consulta de PDFs (backend, frontend y
docker-compose para el volumen de datos).
</commit_message>
<xml_diff>
--- a/app/resources/plantilla_registro.xlsx
+++ b/app/resources/plantilla_registro.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="FORMATO_VENTAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="FORMATO_ COMPRAS " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORMATO_VENTAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORMATO_ COMPRAS " sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>